<commit_message>
did hands on 3
</commit_message>
<xml_diff>
--- a/HandsOn3/Summary.xlsx
+++ b/HandsOn3/Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\HIT\IOT\HandsOn3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F393C42-05B5-4849-8EAA-EAFCAB9D39F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B35679-C4A5-411A-8C2B-BC69E39EB502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26475" yWindow="2565" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31170" yWindow="2385" windowWidth="21600" windowHeight="13920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -471,7 +471,9 @@
       <c r="E4" s="1">
         <v>1</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="b">
@@ -486,7 +488,9 @@
       <c r="E5" s="1">
         <v>0</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="b">
@@ -501,7 +505,9 @@
       <c r="E6" s="1">
         <v>1</v>
       </c>
-      <c r="F6" s="1"/>
+      <c r="F6" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="b">
@@ -516,7 +522,9 @@
       <c r="E7" s="1">
         <v>0</v>
       </c>
-      <c r="F7" s="1"/>
+      <c r="F7" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="b">
@@ -531,7 +539,9 @@
       <c r="E8" s="1">
         <v>1</v>
       </c>
-      <c r="F8" s="1"/>
+      <c r="F8" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="b">
@@ -546,7 +556,9 @@
       <c r="E9" s="1">
         <v>0</v>
       </c>
-      <c r="F9" s="1"/>
+      <c r="F9" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="b">
@@ -561,7 +573,9 @@
       <c r="E10" s="1">
         <v>1</v>
       </c>
-      <c r="F10" s="1"/>
+      <c r="F10" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="b">
@@ -576,7 +590,9 @@
       <c r="E11" s="1">
         <v>0</v>
       </c>
-      <c r="F11" s="1"/>
+      <c r="F11" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="b">
@@ -591,7 +607,9 @@
       <c r="E12" s="1">
         <v>1</v>
       </c>
-      <c r="F12" s="1"/>
+      <c r="F12" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="b">
@@ -606,7 +624,9 @@
       <c r="E13" s="1">
         <v>0</v>
       </c>
-      <c r="F13" s="1"/>
+      <c r="F13" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="b">
@@ -621,7 +641,9 @@
       <c r="E14" s="1">
         <v>1</v>
       </c>
-      <c r="F14" s="1"/>
+      <c r="F14" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="b">
@@ -636,7 +658,9 @@
       <c r="E15" s="1">
         <v>0</v>
       </c>
-      <c r="F15" s="1"/>
+      <c r="F15" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="b">
@@ -651,7 +675,9 @@
       <c r="E16" s="1">
         <v>1</v>
       </c>
-      <c r="F16" s="1"/>
+      <c r="F16" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="b">
@@ -666,7 +692,9 @@
       <c r="E17" s="1">
         <v>0</v>
       </c>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="b">
@@ -681,7 +709,9 @@
       <c r="E18" s="1">
         <v>1</v>
       </c>
-      <c r="F18" s="1"/>
+      <c r="F18" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>